<commit_message>
fix: cot tham khao trong mau Excel dem DON thay vi dem DONG
Cot 'So don' dang dem so dong sales_fact (moi don co nhieu dong san pham)
nen lech voi so tren dashboard. Vd 2025-01 hien 3 nhung thuc te 2 don.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MAU-BO-SUNG-CHI-PHI-ADS.xlsx
+++ b/MAU-BO-SUNG-CHI-PHI-ADS.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Số đơn (tham khảo)</t>
+          <t>Số ĐƠN (tham khảo)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
@@ -718,7 +718,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2" s="6" t="n">
         <v>1285200</v>
@@ -738,7 +738,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="D3" s="6" t="n">
         <v>14053000</v>
@@ -758,7 +758,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>33103800</v>
@@ -778,7 +778,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>274</v>
+        <v>158</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>124884500</v>
@@ -798,7 +798,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>287</v>
+        <v>155</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>172853700</v>
@@ -818,7 +818,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>218</v>
+        <v>163</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>145267800</v>
@@ -838,7 +838,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>208</v>
+        <v>190</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>200713208</v>
@@ -858,7 +858,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>168958024</v>
@@ -878,7 +878,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>179145550</v>
@@ -898,7 +898,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>176</v>
+        <v>160</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>236565429</v>
@@ -918,7 +918,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>184</v>
+        <v>141</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>203009905</v>
@@ -938,7 +938,7 @@
         <v>12</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>198</v>
+        <v>167</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>178289695</v>
@@ -958,7 +958,7 @@
         <v>3</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>144</v>
+        <v>108</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>97220876</v>
@@ -970,6 +970,7 @@
       <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="n"/>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>

</xml_diff>